<commit_message>
Master Sep v14: revenue split of 27.10; model review fixes; October CTRL 9+3
- Split input, «Расшифровка» and «Свод общий» replaced with the 27.10 file
- 25 Bridge: corp PL revenue incl. 1C in other income; corp PL -> model
  revenue block showing deals on other directions' RN
- 17 PL предварительный: Rev-month flag by Rev amount; M+ row added
- 13 Для слайда: «Свод общий» lookup by header; other-inventory row;
  control vs GR without M+ row
- 14 Триггеры: scenarios 1-2 use Rev (BiP) regardless of selected scenario
- 22 Загрузка: «ready to close» only when uploads are in place
- README and labels updated
- CTRL vs ACT: October CTRL = 9+3 from v14 with M+ line; September ACT
  by direction from the updated UO (comparable to 8+4, without M+)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TjyVtBMeKRjjZMJmWM6RZp
</commit_message>
<xml_diff>
--- a/CTRL_vs_ACT_AdTech_2026.xlsx
+++ b/CTRL_vs_ACT_AdTech_2026.xlsx
@@ -7336,7 +7336,7 @@
       </c>
       <c r="B4" s="187">
         <f>IF('AdTech Сентябрь'!C5="","",'AdTech Сентябрь'!C5)</f>
-        <v>1183193163.13</v>
+        <v>1183193163.08</v>
       </c>
       <c r="C4" s="91">
         <f>IF(B4="","",B4/B$4)</f>
@@ -7352,7 +7352,7 @@
       </c>
       <c r="F4" s="188">
         <f>IF(B4="","",B4-D4)</f>
-        <v>56992669.7600002</v>
+        <v>56992669.71</v>
       </c>
       <c r="G4" s="93">
         <f>IF(B4="","",C4-E4)</f>
@@ -7368,7 +7368,7 @@
       </c>
       <c r="J4" s="189">
         <f>'AdTech Октябрь'!E5</f>
-        <v>971690946.05</v>
+        <v>1250103996.52</v>
       </c>
       <c r="K4" s="91">
         <f>J4/J$4</f>
@@ -7384,7 +7384,7 @@
       </c>
       <c r="N4" s="189">
         <f>N(B4)+N(H4)</f>
-        <v>1183193163.13</v>
+        <v>1183193163.08</v>
       </c>
       <c r="O4" s="91">
         <f>IF(N4="","",N4/N$4)</f>
@@ -7400,7 +7400,7 @@
       </c>
       <c r="R4" s="190">
         <f>IF(N4="","",N4-P4)</f>
-        <v>56992669.7600002</v>
+        <v>56992669.71</v>
       </c>
       <c r="S4" s="191">
         <f>IF(N4="","",O4-Q4)</f>
@@ -7439,11 +7439,11 @@
       </c>
       <c r="B5" s="192">
         <f>IF('AdTech Сентябрь'!C6="","",'AdTech Сентябрь'!C6)</f>
-        <v>457989994.88</v>
+        <v>467525662.62</v>
       </c>
       <c r="C5" s="97">
         <f>IF(B5="","",B5/B$4)</f>
-        <v>0.387079649504093</v>
+        <v>0.39513891493674</v>
       </c>
       <c r="D5" s="192">
         <f>'AdTech Сентябрь'!E6</f>
@@ -7455,11 +7455,11 @@
       </c>
       <c r="F5" s="193">
         <f>IF(B5="","",B5-D5)</f>
-        <v>-307336610.69</v>
+        <v>-297800942.95</v>
       </c>
       <c r="G5" s="99">
         <f>IF(B5="","",C5-E5)</f>
-        <v>-0.292485499042295</v>
+        <v>-0.284426233609649</v>
       </c>
       <c r="H5" s="194" t="str">
         <f>IF('AdTech Октябрь'!C6="","",'AdTech Октябрь'!C6)</f>
@@ -7471,11 +7471,11 @@
       </c>
       <c r="J5" s="194">
         <f>'AdTech Октябрь'!E6</f>
-        <v>560927053.33</v>
+        <v>561821896.05</v>
       </c>
       <c r="K5" s="97">
         <f>J5/J$4</f>
-        <v>0.577268992378917</v>
+        <v>0.449420126336674</v>
       </c>
       <c r="L5" s="195" t="str">
         <f>IF(H5="","",H5-J5)</f>
@@ -7487,11 +7487,11 @@
       </c>
       <c r="N5" s="194">
         <f>N(B5)+N(H5)</f>
-        <v>457989994.88</v>
+        <v>467525662.62</v>
       </c>
       <c r="O5" s="97">
         <f>IF(N5="","",N5/N$4)</f>
-        <v>0.387079649504093</v>
+        <v>0.39513891493674</v>
       </c>
       <c r="P5" s="194">
         <f>D5+IF(H5="",0,J5)</f>
@@ -7503,11 +7503,11 @@
       </c>
       <c r="R5" s="195">
         <f>IF(N5="","",N5-P5)</f>
-        <v>-307336610.69</v>
+        <v>-297800942.95</v>
       </c>
       <c r="S5" s="196">
         <f>IF(N5="","",O5-Q5)</f>
-        <v>-0.292485499042295</v>
+        <v>-0.284426233609649</v>
       </c>
       <c r="T5" s="181" t="n"/>
       <c r="U5" s="181" t="n"/>
@@ -7578,7 +7578,7 @@
       </c>
       <c r="K6" s="97">
         <f>J6/J$4</f>
-        <v>0.000839942240192493</v>
+        <v>0.000652877098443019</v>
       </c>
       <c r="L6" s="195" t="str">
         <f>IF(H6="","",H6-J6)</f>
@@ -7681,7 +7681,7 @@
       </c>
       <c r="K7" s="102">
         <f>J7/J$4</f>
-        <v>0.000462459253970323</v>
+        <v>0.000359464069590158</v>
       </c>
       <c r="L7" s="195" t="str">
         <f>IF(H7="","",H7-J7)</f>
@@ -7752,7 +7752,7 @@
       </c>
       <c r="C8" s="97">
         <f>IF(B8="","",B8/B$4)</f>
-        <v>0.00205589035315676</v>
+        <v>0.00205589035324364</v>
       </c>
       <c r="D8" s="192">
         <f>'AdTech Сентябрь'!E9</f>
@@ -7768,7 +7768,7 @@
       </c>
       <c r="G8" s="99">
         <f>IF(B8="","",C8-E8)</f>
-        <v>-0.00226125283637535</v>
+        <v>-0.00226125283628847</v>
       </c>
       <c r="H8" s="194" t="str">
         <f>IF('AdTech Октябрь'!C9="","",'AdTech Октябрь'!C9)</f>
@@ -7784,7 +7784,7 @@
       </c>
       <c r="K8" s="97">
         <f>J8/J$4</f>
-        <v>0.0051554321673614</v>
+        <v>0.00400725601545572</v>
       </c>
       <c r="L8" s="195" t="str">
         <f>IF(H8="","",H8-J8)</f>
@@ -7800,7 +7800,7 @@
       </c>
       <c r="O8" s="97">
         <f>IF(N8="","",N8/N$4)</f>
-        <v>0.00205589035315676</v>
+        <v>0.00205589035324364</v>
       </c>
       <c r="P8" s="194">
         <f>D8+IF(H8="",0,J8)</f>
@@ -7816,7 +7816,7 @@
       </c>
       <c r="S8" s="196">
         <f>IF(N8="","",O8-Q8)</f>
-        <v>-0.00226125283637535</v>
+        <v>-0.00226125283628847</v>
       </c>
       <c r="T8" s="181" t="n"/>
       <c r="U8" s="181" t="n"/>
@@ -7855,7 +7855,7 @@
       </c>
       <c r="C9" s="97">
         <f>IF(B9="","",B9/B$4)</f>
-        <v>0.170445289217617</v>
+        <v>0.17044528922482</v>
       </c>
       <c r="D9" s="192">
         <f>'AdTech Сентябрь'!E10</f>
@@ -7871,7 +7871,7 @@
       </c>
       <c r="G9" s="99">
         <f>IF(B9="","",C9-E9)</f>
-        <v>0.108751493673191</v>
+        <v>0.108751493680394</v>
       </c>
       <c r="H9" s="194" t="str">
         <f>IF('AdTech Октябрь'!C10="","",'AdTech Октябрь'!C10)</f>
@@ -7887,7 +7887,7 @@
       </c>
       <c r="K9" s="97">
         <f>J9/J$4</f>
-        <v>0.0944939887247599</v>
+        <v>0.0734490518833655</v>
       </c>
       <c r="L9" s="195" t="str">
         <f>IF(H9="","",H9-J9)</f>
@@ -7903,7 +7903,7 @@
       </c>
       <c r="O9" s="97">
         <f>IF(N9="","",N9/N$4)</f>
-        <v>0.170445289217617</v>
+        <v>0.17044528922482</v>
       </c>
       <c r="P9" s="194">
         <f>D9+IF(H9="",0,J9)</f>
@@ -7919,7 +7919,7 @@
       </c>
       <c r="S9" s="196">
         <f>IF(N9="","",O9-Q9)</f>
-        <v>0.108751493673191</v>
+        <v>0.108751493680394</v>
       </c>
       <c r="T9" s="181" t="n"/>
       <c r="U9" s="181" t="n"/>
@@ -7954,11 +7954,11 @@
       </c>
       <c r="B10" s="192">
         <f>IF('AdTech Сентябрь'!C11="","",'AdTech Сентябрь'!C11)</f>
-        <v>421805564.12</v>
+        <v>413469896.39</v>
       </c>
       <c r="C10" s="97">
         <f>IF(B10="","",B10/B$4)</f>
-        <v>0.35649763475996</v>
+        <v>0.349452574010558</v>
       </c>
       <c r="D10" s="192">
         <f>'AdTech Сентябрь'!E11</f>
@@ -7970,11 +7970,11 @@
       </c>
       <c r="F10" s="193">
         <f>IF(B10="","",B10-D10)</f>
-        <v>260428357.69</v>
+        <v>252092689.96</v>
       </c>
       <c r="G10" s="99">
         <f>IF(B10="","",C10-E10)</f>
-        <v>0.213204138282169</v>
+        <v>0.206159077532768</v>
       </c>
       <c r="H10" s="194" t="str">
         <f>IF('AdTech Октябрь'!C11="","",'AdTech Октябрь'!C11)</f>
@@ -7990,7 +7990,7 @@
       </c>
       <c r="K10" s="97">
         <f>J10/J$4</f>
-        <v>0.27056728833251</v>
+        <v>0.210308730395131</v>
       </c>
       <c r="L10" s="195" t="str">
         <f>IF(H10="","",H10-J10)</f>
@@ -8002,11 +8002,11 @@
       </c>
       <c r="N10" s="194">
         <f>N(B10)+N(H10)</f>
-        <v>421805564.12</v>
+        <v>413469896.39</v>
       </c>
       <c r="O10" s="97">
         <f>IF(N10="","",N10/N$4)</f>
-        <v>0.35649763475996</v>
+        <v>0.349452574010558</v>
       </c>
       <c r="P10" s="194">
         <f>D10+IF(H10="",0,J10)</f>
@@ -8018,11 +8018,11 @@
       </c>
       <c r="R10" s="195">
         <f>IF(N10="","",N10-P10)</f>
-        <v>260428357.69</v>
+        <v>252092689.96</v>
       </c>
       <c r="S10" s="196">
         <f>IF(N10="","",O10-Q10)</f>
-        <v>0.213204138282169</v>
+        <v>0.206159077532768</v>
       </c>
       <c r="T10" s="181" t="n"/>
       <c r="U10" s="181" t="n"/>
@@ -8093,7 +8093,7 @@
       </c>
       <c r="K11" s="97">
         <f>J11/J$4</f>
-        <v>0.048464191028468</v>
+        <v>0.0376706384117592</v>
       </c>
       <c r="L11" s="195" t="str">
         <f>IF(H11="","",H11-J11)</f>
@@ -8164,7 +8164,7 @@
       </c>
       <c r="C12" s="97">
         <f>IF(B12="","",B12/B$4)</f>
-        <v>0.000385584657025164</v>
+        <v>0.000385584657041458</v>
       </c>
       <c r="D12" s="192">
         <f>'AdTech Сентябрь'!E13</f>
@@ -8180,7 +8180,7 @@
       </c>
       <c r="G12" s="99">
         <f>IF(B12="","",C12-E12)</f>
-        <v>-0.00185011602400161</v>
+        <v>-0.00185011602398532</v>
       </c>
       <c r="H12" s="194" t="str">
         <f>IF('AdTech Октябрь'!C13="","",'AdTech Октябрь'!C13)</f>
@@ -8196,7 +8196,7 @@
       </c>
       <c r="K12" s="97">
         <f>J12/J$4</f>
-        <v>0.00274770587382072</v>
+        <v>0.00213575904679326</v>
       </c>
       <c r="L12" s="195" t="str">
         <f>IF(H12="","",H12-J12)</f>
@@ -8212,7 +8212,7 @@
       </c>
       <c r="O12" s="97">
         <f>IF(N12="","",N12/N$4)</f>
-        <v>0.000385584657025164</v>
+        <v>0.000385584657041458</v>
       </c>
       <c r="P12" s="194">
         <f>D12+IF(H12="",0,J12)</f>
@@ -8228,7 +8228,7 @@
       </c>
       <c r="S12" s="196">
         <f>IF(N12="","",O12-Q12)</f>
-        <v>-0.00185011602400161</v>
+        <v>-0.00185011602398532</v>
       </c>
       <c r="T12" s="181" t="n"/>
       <c r="U12" s="181" t="n"/>
@@ -8267,7 +8267,7 @@
       </c>
       <c r="C13" s="97">
         <f>IF(B13="","",B13/B$4)</f>
-        <v>0.0801321377222857</v>
+        <v>0.080132137725672</v>
       </c>
       <c r="D13" s="192">
         <f>'AdTech Сентябрь'!E14</f>
@@ -8283,7 +8283,7 @@
       </c>
       <c r="G13" s="99">
         <f>IF(B13="","",C13-E13)</f>
-        <v>0.0801321377222857</v>
+        <v>0.080132137725672</v>
       </c>
       <c r="H13" s="194" t="str">
         <f>IF('AdTech Октябрь'!C14="","",'AdTech Октябрь'!C14)</f>
@@ -8315,7 +8315,7 @@
       </c>
       <c r="O13" s="97">
         <f>IF(N13="","",N13/N$4)</f>
-        <v>0.0801321377222857</v>
+        <v>0.080132137725672</v>
       </c>
       <c r="P13" s="194">
         <f>D13+IF(H13="",0,J13)</f>
@@ -8331,7 +8331,7 @@
       </c>
       <c r="S13" s="196">
         <f>IF(N13="","",O13-Q13)</f>
-        <v>0.0801321377222857</v>
+        <v>0.080132137725672</v>
       </c>
       <c r="T13" s="181" t="n"/>
       <c r="U13" s="181" t="n"/>
@@ -8366,11 +8366,11 @@
       </c>
       <c r="B14" s="192">
         <f>IF('AdTech Сентябрь'!C15="","",'AdTech Сентябрь'!C15)</f>
-        <v>4027369.15</v>
+        <v>2827369.14</v>
       </c>
       <c r="C14" s="97">
         <f>IF(B14="","",B14/B$4)</f>
-        <v>0.00340381374360384</v>
+        <v>0.00238960909192545</v>
       </c>
       <c r="D14" s="192">
         <f>'AdTech Сентябрь'!E15</f>
@@ -8382,11 +8382,11 @@
       </c>
       <c r="F14" s="193">
         <f>IF(B14="","",B14-D14)</f>
-        <v>4027369.15</v>
+        <v>2827369.14</v>
       </c>
       <c r="G14" s="99">
         <f>IF(B14="","",C14-E14)</f>
-        <v>0.00340381374360384</v>
+        <v>0.00238960909192545</v>
       </c>
       <c r="H14" s="194" t="str">
         <f>IF('AdTech Октябрь'!C15="","",'AdTech Октябрь'!C15)</f>
@@ -8414,11 +8414,11 @@
       </c>
       <c r="N14" s="194">
         <f>N(B14)+N(H14)</f>
-        <v>4027369.15</v>
+        <v>2827369.14</v>
       </c>
       <c r="O14" s="97">
         <f>IF(N14="","",N14/N$4)</f>
-        <v>0.00340381374360384</v>
+        <v>0.00238960909192545</v>
       </c>
       <c r="P14" s="194">
         <f>D14+IF(H14="",0,J14)</f>
@@ -8430,11 +8430,11 @@
       </c>
       <c r="R14" s="195">
         <f>IF(N14="","",N14-P14)</f>
-        <v>4027369.15</v>
+        <v>2827369.14</v>
       </c>
       <c r="S14" s="196">
         <f>IF(N14="","",O14-Q14)</f>
-        <v>0.00340381374360384</v>
+        <v>0.00238960909192545</v>
       </c>
       <c r="T14" s="181" t="n"/>
       <c r="U14" s="181" t="n"/>
@@ -8464,32 +8464,32 @@
     <row r="15" ht="17.5" customHeight="1" s="12">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Direct cost</t>
+          <t>М+ и сверка со сплитом</t>
         </is>
       </c>
       <c r="B15" s="192">
         <f>IF('AdTech Сентябрь'!C16="","",'AdTech Сентябрь'!C16)</f>
-        <v>-927852.26</v>
+        <v>0</v>
       </c>
       <c r="C15" s="97">
         <f>IF(B15="","",B15/B$4)</f>
-        <v>-0.000784193392011728</v>
+        <v>0</v>
       </c>
       <c r="D15" s="192">
         <f>'AdTech Сентябрь'!E16</f>
-        <v>-34765800.63</v>
+        <v>0</v>
       </c>
       <c r="E15" s="97">
         <f>D15/D$4</f>
-        <v>-0.0308699923634096</v>
+        <v>0</v>
       </c>
       <c r="F15" s="193">
         <f>IF(B15="","",B15-D15)</f>
-        <v>33837948.37</v>
+        <v>0</v>
       </c>
       <c r="G15" s="99">
         <f>IF(B15="","",C15-E15)</f>
-        <v>0.0300857989713979</v>
+        <v>0</v>
       </c>
       <c r="H15" s="194" t="str">
         <f>IF('AdTech Октябрь'!C16="","",'AdTech Октябрь'!C16)</f>
@@ -8501,11 +8501,11 @@
       </c>
       <c r="J15" s="194">
         <f>'AdTech Октябрь'!E16</f>
-        <v>-37708031.15</v>
+        <v>277518207.76</v>
       </c>
       <c r="K15" s="97">
         <f>J15/J$4</f>
-        <v>-0.0388066095534657</v>
+        <v>0.221996096750787</v>
       </c>
       <c r="L15" s="195" t="str">
         <f>IF(H15="","",H15-J15)</f>
@@ -8517,27 +8517,27 @@
       </c>
       <c r="N15" s="194">
         <f>N(B15)+N(H15)</f>
-        <v>-927852.26</v>
+        <v>0</v>
       </c>
       <c r="O15" s="97">
         <f>IF(N15="","",N15/N$4)</f>
-        <v>-0.000784193392011728</v>
+        <v>0</v>
       </c>
       <c r="P15" s="194">
         <f>D15+IF(H15="",0,J15)</f>
-        <v>-34765800.63</v>
+        <v>0</v>
       </c>
       <c r="Q15" s="97">
         <f>P15/P$4</f>
-        <v>-0.0308699923634096</v>
+        <v>0</v>
       </c>
       <c r="R15" s="195">
         <f>IF(N15="","",N15-P15)</f>
-        <v>33837948.37</v>
+        <v>0</v>
       </c>
       <c r="S15" s="196">
         <f>IF(N15="","",O15-Q15)</f>
-        <v>0.0300857989713979</v>
+        <v>0</v>
       </c>
       <c r="T15" s="181" t="n"/>
       <c r="U15" s="181" t="n"/>
@@ -8567,32 +8567,32 @@
     <row r="16" ht="17.5" customHeight="1" s="12">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>PEX</t>
+          <t>Direct cost</t>
         </is>
       </c>
       <c r="B16" s="192">
         <f>IF('AdTech Сентябрь'!C17="","",'AdTech Сентябрь'!C17)</f>
-        <v>62456405.7</v>
+        <v>-927852.26</v>
       </c>
       <c r="C16" s="97">
         <f>IF(B16="","",B16/B$4)</f>
-        <v>0.0527863138887473</v>
+        <v>-0.000784193392044867</v>
       </c>
       <c r="D16" s="192">
         <f>'AdTech Сентябрь'!E17</f>
-        <v>-111510282.75</v>
+        <v>-34765800.63</v>
       </c>
       <c r="E16" s="97">
         <f>D16/D$4</f>
-        <v>-0.0990145923452056</v>
+        <v>-0.0308699923634096</v>
       </c>
       <c r="F16" s="193">
         <f>IF(B16="","",B16-D16)</f>
-        <v>173966688.45</v>
+        <v>33837948.37</v>
       </c>
       <c r="G16" s="99">
         <f>IF(B16="","",C16-E16)</f>
-        <v>0.151800906233953</v>
+        <v>0.0300857989713647</v>
       </c>
       <c r="H16" s="194" t="str">
         <f>IF('AdTech Октябрь'!C17="","",'AdTech Октябрь'!C17)</f>
@@ -8604,11 +8604,11 @@
       </c>
       <c r="J16" s="194">
         <f>'AdTech Октябрь'!E17</f>
-        <v>-89694325.25</v>
+        <v>-37791001.81</v>
       </c>
       <c r="K16" s="97">
         <f>J16/J$4</f>
-        <v>-0.0923074621767492</v>
+        <v>-0.0302302863723349</v>
       </c>
       <c r="L16" s="195" t="str">
         <f>IF(H16="","",H16-J16)</f>
@@ -8620,27 +8620,27 @@
       </c>
       <c r="N16" s="194">
         <f>N(B16)+N(H16)</f>
-        <v>62456405.7</v>
+        <v>-927852.26</v>
       </c>
       <c r="O16" s="97">
         <f>IF(N16="","",N16/N$4)</f>
-        <v>0.0527863138887473</v>
+        <v>-0.000784193392044867</v>
       </c>
       <c r="P16" s="194">
         <f>D16+IF(H16="",0,J16)</f>
-        <v>-111510282.75</v>
+        <v>-34765800.63</v>
       </c>
       <c r="Q16" s="97">
         <f>P16/P$4</f>
-        <v>-0.0990145923452056</v>
+        <v>-0.0308699923634096</v>
       </c>
       <c r="R16" s="195">
         <f>IF(N16="","",N16-P16)</f>
-        <v>173966688.45</v>
+        <v>33837948.37</v>
       </c>
       <c r="S16" s="196">
         <f>IF(N16="","",O16-Q16)</f>
-        <v>0.151800906233953</v>
+        <v>0.0300857989713647</v>
       </c>
       <c r="T16" s="181" t="n"/>
       <c r="U16" s="181" t="n"/>
@@ -8670,32 +8670,32 @@
     <row r="17" ht="17.5" customHeight="1" s="12">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Other PEX</t>
+          <t>PEX</t>
         </is>
       </c>
       <c r="B17" s="192">
         <f>IF('AdTech Сентябрь'!C18="","",'AdTech Сентябрь'!C18)</f>
-        <v>-211306.16</v>
+        <v>62456405.7</v>
       </c>
       <c r="C17" s="97">
         <f>IF(B17="","",B17/B$4)</f>
-        <v>-0.000178589740529783</v>
+        <v>0.052786313890978</v>
       </c>
       <c r="D17" s="192">
         <f>'AdTech Сентябрь'!E18</f>
-        <v>-4338633.91</v>
+        <v>-111510282.75</v>
       </c>
       <c r="E17" s="97">
         <f>D17/D$4</f>
-        <v>-0.00385245250338795</v>
+        <v>-0.0990145923452056</v>
       </c>
       <c r="F17" s="193">
         <f>IF(B17="","",B17-D17)</f>
-        <v>4127327.75</v>
+        <v>173966688.45</v>
       </c>
       <c r="G17" s="99">
         <f>IF(B17="","",C17-E17)</f>
-        <v>0.00367386276285817</v>
+        <v>0.151800906236184</v>
       </c>
       <c r="H17" s="194" t="str">
         <f>IF('AdTech Октябрь'!C18="","",'AdTech Октябрь'!C18)</f>
@@ -8707,11 +8707,11 @@
       </c>
       <c r="J17" s="194">
         <f>'AdTech Октябрь'!E18</f>
-        <v>-5807323.07</v>
+        <v>-89694325.25</v>
       </c>
       <c r="K17" s="97">
         <f>J17/J$4</f>
-        <v>-0.00597651248435238</v>
+        <v>-0.0717494908421125</v>
       </c>
       <c r="L17" s="195" t="str">
         <f>IF(H17="","",H17-J17)</f>
@@ -8723,27 +8723,27 @@
       </c>
       <c r="N17" s="194">
         <f>N(B17)+N(H17)</f>
-        <v>-211306.16</v>
+        <v>62456405.7</v>
       </c>
       <c r="O17" s="97">
         <f>IF(N17="","",N17/N$4)</f>
-        <v>-0.000178589740529783</v>
+        <v>0.052786313890978</v>
       </c>
       <c r="P17" s="194">
         <f>D17+IF(H17="",0,J17)</f>
-        <v>-4338633.91</v>
+        <v>-111510282.75</v>
       </c>
       <c r="Q17" s="97">
         <f>P17/P$4</f>
-        <v>-0.00385245250338795</v>
+        <v>-0.0990145923452056</v>
       </c>
       <c r="R17" s="195">
         <f>IF(N17="","",N17-P17)</f>
-        <v>4127327.75</v>
+        <v>173966688.45</v>
       </c>
       <c r="S17" s="196">
         <f>IF(N17="","",O17-Q17)</f>
-        <v>0.00367386276285817</v>
+        <v>0.151800906236184</v>
       </c>
       <c r="T17" s="181" t="n"/>
       <c r="U17" s="181" t="n"/>
@@ -8773,32 +8773,32 @@
     <row r="18" ht="17.5" customHeight="1" s="12">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Other PEX</t>
         </is>
       </c>
       <c r="B18" s="192">
         <f>IF('AdTech Сентябрь'!C19="","",'AdTech Сентябрь'!C19)</f>
-        <v>-105089188</v>
+        <v>-211306.16</v>
       </c>
       <c r="C18" s="97">
         <f>IF(B18="","",B18/B$4)</f>
-        <v>-0.0888182853609454</v>
+        <v>-0.00017858974053733</v>
       </c>
       <c r="D18" s="192">
         <f>'AdTech Сентябрь'!E19</f>
-        <v>-348750338.14</v>
+        <v>-4338633.91</v>
       </c>
       <c r="E18" s="97">
         <f>D18/D$4</f>
-        <v>-0.309669850255892</v>
+        <v>-0.00385245250338795</v>
       </c>
       <c r="F18" s="193">
         <f>IF(B18="","",B18-D18)</f>
-        <v>243661150.14</v>
+        <v>4127327.75</v>
       </c>
       <c r="G18" s="99">
         <f>IF(B18="","",C18-E18)</f>
-        <v>0.220851564894947</v>
+        <v>0.00367386276285062</v>
       </c>
       <c r="H18" s="194" t="str">
         <f>IF('AdTech Октябрь'!C19="","",'AdTech Октябрь'!C19)</f>
@@ -8810,11 +8810,11 @@
       </c>
       <c r="J18" s="194">
         <f>'AdTech Октябрь'!E19</f>
-        <v>-101498947.99</v>
+        <v>-5807323.07</v>
       </c>
       <c r="K18" s="97">
         <f>J18/J$4</f>
-        <v>-0.104455998486557</v>
+        <v>-0.00464547196566545</v>
       </c>
       <c r="L18" s="195" t="str">
         <f>IF(H18="","",H18-J18)</f>
@@ -8826,27 +8826,27 @@
       </c>
       <c r="N18" s="194">
         <f>N(B18)+N(H18)</f>
-        <v>-105089188</v>
+        <v>-211306.16</v>
       </c>
       <c r="O18" s="97">
         <f>IF(N18="","",N18/N$4)</f>
-        <v>-0.0888182853609454</v>
+        <v>-0.00017858974053733</v>
       </c>
       <c r="P18" s="194">
         <f>D18+IF(H18="",0,J18)</f>
-        <v>-348750338.14</v>
+        <v>-4338633.91</v>
       </c>
       <c r="Q18" s="97">
         <f>P18/P$4</f>
-        <v>-0.309669850255892</v>
+        <v>-0.00385245250338795</v>
       </c>
       <c r="R18" s="195">
         <f>IF(N18="","",N18-P18)</f>
-        <v>243661150.14</v>
+        <v>4127327.75</v>
       </c>
       <c r="S18" s="196">
         <f>IF(N18="","",O18-Q18)</f>
-        <v>0.220851564894947</v>
+        <v>0.00367386276285062</v>
       </c>
       <c r="T18" s="181" t="n"/>
       <c r="U18" s="181" t="n"/>
@@ -8876,32 +8876,32 @@
     <row r="19" ht="17.5" customHeight="1" s="12">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="B19" s="192">
         <f>IF('AdTech Сентябрь'!C20="","",'AdTech Сентябрь'!C20)</f>
-        <v>-3887514.7</v>
+        <v>-105089188</v>
       </c>
       <c r="C19" s="97">
         <f>IF(B19="","",B19/B$4)</f>
-        <v>-0.00328561288312048</v>
+        <v>-0.0888182853646988</v>
       </c>
       <c r="D19" s="192">
         <f>'AdTech Сентябрь'!E20</f>
-        <v>-1283507.24</v>
+        <v>-348750338.14</v>
       </c>
       <c r="E19" s="97">
         <f>D19/D$4</f>
-        <v>-0.0011396791668589</v>
+        <v>-0.309669850255892</v>
       </c>
       <c r="F19" s="193">
         <f>IF(B19="","",B19-D19)</f>
-        <v>-2604007.46</v>
+        <v>243661150.14</v>
       </c>
       <c r="G19" s="99">
         <f>IF(B19="","",C19-E19)</f>
-        <v>-0.00214593371626158</v>
+        <v>0.220851564891194</v>
       </c>
       <c r="H19" s="194" t="str">
         <f>IF('AdTech Октябрь'!C20="","",'AdTech Октябрь'!C20)</f>
@@ -8913,11 +8913,11 @@
       </c>
       <c r="J19" s="194">
         <f>'AdTech Октябрь'!E20</f>
-        <v>-1857987.23</v>
+        <v>-101647328.58</v>
       </c>
       <c r="K19" s="97">
         <f>J19/J$4</f>
-        <v>-0.00191211746651841</v>
+        <v>-0.0813110980070159</v>
       </c>
       <c r="L19" s="195" t="str">
         <f>IF(H19="","",H19-J19)</f>
@@ -8929,27 +8929,27 @@
       </c>
       <c r="N19" s="194">
         <f>N(B19)+N(H19)</f>
-        <v>-3887514.7</v>
+        <v>-105089188</v>
       </c>
       <c r="O19" s="97">
         <f>IF(N19="","",N19/N$4)</f>
-        <v>-0.00328561288312048</v>
+        <v>-0.0888182853646988</v>
       </c>
       <c r="P19" s="194">
         <f>D19+IF(H19="",0,J19)</f>
-        <v>-1283507.24</v>
+        <v>-348750338.14</v>
       </c>
       <c r="Q19" s="97">
         <f>P19/P$4</f>
-        <v>-0.0011396791668589</v>
+        <v>-0.309669850255892</v>
       </c>
       <c r="R19" s="195">
         <f>IF(N19="","",N19-P19)</f>
-        <v>-2604007.46</v>
+        <v>243661150.14</v>
       </c>
       <c r="S19" s="196">
         <f>IF(N19="","",O19-Q19)</f>
-        <v>-0.00214593371626158</v>
+        <v>0.220851564891194</v>
       </c>
       <c r="T19" s="181" t="n"/>
       <c r="U19" s="181" t="n"/>
@@ -8979,32 +8979,32 @@
     <row r="20" ht="17.5" customHeight="1" s="12">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Other OPEX</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="B20" s="192">
         <f>IF('AdTech Сентябрь'!C21="","",'AdTech Сентябрь'!C21)</f>
-        <v>-9123175.28</v>
+        <v>-3887514.7</v>
       </c>
       <c r="C20" s="97">
         <f>IF(B20="","",B20/B$4)</f>
-        <v>-0.00771063894239018</v>
+        <v>-0.00328561288325933</v>
       </c>
       <c r="D20" s="192">
         <f>'AdTech Сентябрь'!E21</f>
-        <v>-5047284.06</v>
+        <v>-1283507.24</v>
       </c>
       <c r="E20" s="97">
         <f>D20/D$4</f>
-        <v>-0.00448169228278057</v>
+        <v>-0.0011396791668589</v>
       </c>
       <c r="F20" s="193">
         <f>IF(B20="","",B20-D20)</f>
-        <v>-4075891.22</v>
+        <v>-2604007.46</v>
       </c>
       <c r="G20" s="99">
         <f>IF(B20="","",C20-E20)</f>
-        <v>-0.00322894665960961</v>
+        <v>-0.00214593371640043</v>
       </c>
       <c r="H20" s="194" t="str">
         <f>IF('AdTech Октябрь'!C21="","",'AdTech Октябрь'!C21)</f>
@@ -9016,11 +9016,11 @@
       </c>
       <c r="J20" s="194">
         <f>'AdTech Октябрь'!E21</f>
-        <v>-5649652.71</v>
+        <v>-1857987.23</v>
       </c>
       <c r="K20" s="97">
         <f>J20/J$4</f>
-        <v>-0.005814248586926</v>
+        <v>-0.00148626613079568</v>
       </c>
       <c r="L20" s="195" t="str">
         <f>IF(H20="","",H20-J20)</f>
@@ -9032,27 +9032,27 @@
       </c>
       <c r="N20" s="194">
         <f>N(B20)+N(H20)</f>
-        <v>-9123175.28</v>
+        <v>-3887514.7</v>
       </c>
       <c r="O20" s="97">
         <f>IF(N20="","",N20/N$4)</f>
-        <v>-0.00771063894239018</v>
+        <v>-0.00328561288325933</v>
       </c>
       <c r="P20" s="194">
         <f>D20+IF(H20="",0,J20)</f>
-        <v>-5047284.06</v>
+        <v>-1283507.24</v>
       </c>
       <c r="Q20" s="97">
         <f>P20/P$4</f>
-        <v>-0.00448169228278057</v>
+        <v>-0.0011396791668589</v>
       </c>
       <c r="R20" s="195">
         <f>IF(N20="","",N20-P20)</f>
-        <v>-4075891.22</v>
+        <v>-2604007.46</v>
       </c>
       <c r="S20" s="196">
         <f>IF(N20="","",O20-Q20)</f>
-        <v>-0.00322894665960961</v>
+        <v>-0.00214593371640043</v>
       </c>
       <c r="T20" s="181" t="n"/>
       <c r="U20" s="181" t="n"/>
@@ -9080,82 +9080,82 @@
       <c r="AQ20" s="181" t="n"/>
     </row>
     <row r="21" ht="17.5" customHeight="1" s="12">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>EBITDA</t>
-        </is>
-      </c>
-      <c r="B21" s="199">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Other OPEX</t>
+        </is>
+      </c>
+      <c r="B21" s="192">
         <f>IF('AdTech Сентябрь'!C22="","",'AdTech Сентябрь'!C22)</f>
-        <v>1126410532.43</v>
-      </c>
-      <c r="C21" s="109">
+        <v>-9123175.28</v>
+      </c>
+      <c r="C21" s="97">
         <f>IF(B21="","",B21/B$4)</f>
-        <v>0.95200899356975</v>
-      </c>
-      <c r="D21" s="199">
+        <v>-0.00771063894271603</v>
+      </c>
+      <c r="D21" s="192">
         <f>'AdTech Сентябрь'!E22</f>
-        <v>620504646.64</v>
-      </c>
-      <c r="E21" s="109">
+        <v>-5047284.06</v>
+      </c>
+      <c r="E21" s="97">
         <f>D21/D$4</f>
-        <v>0.550971741082465</v>
-      </c>
-      <c r="F21" s="200">
+        <v>-0.00448169228278057</v>
+      </c>
+      <c r="F21" s="193">
         <f>IF(B21="","",B21-D21)</f>
-        <v>505905885.79</v>
-      </c>
-      <c r="G21" s="111">
+        <v>-4075891.22</v>
+      </c>
+      <c r="G21" s="99">
         <f>IF(B21="","",C21-E21)</f>
-        <v>0.401037252487285</v>
-      </c>
-      <c r="H21" s="201" t="str">
+        <v>-0.00322894665993545</v>
+      </c>
+      <c r="H21" s="194" t="str">
         <f>IF('AdTech Октябрь'!C22="","",'AdTech Октябрь'!C22)</f>
         <v/>
       </c>
-      <c r="I21" s="109" t="str">
+      <c r="I21" s="97" t="str">
         <f>IF(H21="","",H21/H$4)</f>
         <v/>
       </c>
-      <c r="J21" s="201">
+      <c r="J21" s="194">
         <f>'AdTech Октябрь'!E22</f>
-        <v>729474678.65</v>
-      </c>
-      <c r="K21" s="109">
+        <v>-5915678.59</v>
+      </c>
+      <c r="K21" s="97">
         <f>J21/J$4</f>
-        <v>0.750727051245431</v>
-      </c>
-      <c r="L21" s="202" t="str">
+        <v>-0.00473214917036333</v>
+      </c>
+      <c r="L21" s="195" t="str">
         <f>IF(H21="","",H21-J21)</f>
         <v/>
       </c>
-      <c r="M21" s="203" t="str">
+      <c r="M21" s="196" t="str">
         <f>IF(H21="","",I21-K21)</f>
         <v/>
       </c>
-      <c r="N21" s="201">
+      <c r="N21" s="194">
         <f>N(B21)+N(H21)</f>
-        <v>1126410532.43</v>
-      </c>
-      <c r="O21" s="109">
+        <v>-9123175.28</v>
+      </c>
+      <c r="O21" s="97">
         <f>IF(N21="","",N21/N$4)</f>
-        <v>0.95200899356975</v>
-      </c>
-      <c r="P21" s="201">
+        <v>-0.00771063894271603</v>
+      </c>
+      <c r="P21" s="194">
         <f>D21+IF(H21="",0,J21)</f>
-        <v>620504646.64</v>
-      </c>
-      <c r="Q21" s="109">
+        <v>-5047284.06</v>
+      </c>
+      <c r="Q21" s="97">
         <f>P21/P$4</f>
-        <v>0.550971741082465</v>
-      </c>
-      <c r="R21" s="202">
+        <v>-0.00448169228278057</v>
+      </c>
+      <c r="R21" s="195">
         <f>IF(N21="","",N21-P21)</f>
-        <v>505905885.79</v>
-      </c>
-      <c r="S21" s="203">
+        <v>-4075891.22</v>
+      </c>
+      <c r="S21" s="196">
         <f>IF(N21="","",O21-Q21)</f>
-        <v>0.401037252487285</v>
+        <v>-0.00322894665993545</v>
       </c>
       <c r="T21" s="181" t="n"/>
       <c r="U21" s="181" t="n"/>
@@ -9183,25 +9183,83 @@
       <c r="AQ21" s="181" t="n"/>
     </row>
     <row r="22" ht="17.5" customHeight="1" s="12">
-      <c r="A22" s="181" t="n"/>
-      <c r="B22" s="181" t="n"/>
-      <c r="C22" s="181" t="n"/>
-      <c r="D22" s="181" t="n"/>
-      <c r="E22" s="181" t="n"/>
-      <c r="F22" s="181" t="n"/>
-      <c r="G22" s="181" t="n"/>
-      <c r="H22" s="181" t="n"/>
-      <c r="I22" s="181" t="n"/>
-      <c r="J22" s="181" t="n"/>
-      <c r="K22" s="181" t="n"/>
-      <c r="L22" s="181" t="n"/>
-      <c r="M22" s="181" t="n"/>
-      <c r="N22" s="181" t="n"/>
-      <c r="O22" s="181" t="n"/>
-      <c r="P22" s="181" t="n"/>
-      <c r="Q22" s="181" t="n"/>
-      <c r="R22" s="181" t="n"/>
-      <c r="S22" s="181" t="n"/>
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="B22" s="199">
+        <f>IF('AdTech Сентябрь'!C23="","",'AdTech Сентябрь'!C23)</f>
+        <v>1126410532.38</v>
+      </c>
+      <c r="C22" s="109">
+        <f>IF(B22="","",B22/B$4)</f>
+        <v>0.952008993567722</v>
+      </c>
+      <c r="D22" s="199">
+        <f>'AdTech Сентябрь'!E23</f>
+        <v>620504646.64</v>
+      </c>
+      <c r="E22" s="109">
+        <f>D22/D$4</f>
+        <v>0.550971741082465</v>
+      </c>
+      <c r="F22" s="200">
+        <f>IF(B22="","",B22-D22)</f>
+        <v>505905885.74</v>
+      </c>
+      <c r="G22" s="111">
+        <f>IF(B22="","",C22-E22)</f>
+        <v>0.401037252485257</v>
+      </c>
+      <c r="H22" s="201" t="str">
+        <f>IF('AdTech Октябрь'!C23="","",'AdTech Октябрь'!C23)</f>
+        <v/>
+      </c>
+      <c r="I22" s="109" t="str">
+        <f>IF(H22="","",H22/H$4)</f>
+        <v/>
+      </c>
+      <c r="J22" s="201">
+        <f>'AdTech Октябрь'!E23</f>
+        <v>1007390351.99</v>
+      </c>
+      <c r="K22" s="109">
+        <f>J22/J$4</f>
+        <v>0.805845237511712</v>
+      </c>
+      <c r="L22" s="202" t="str">
+        <f>IF(H22="","",H22-J22)</f>
+        <v/>
+      </c>
+      <c r="M22" s="203" t="str">
+        <f>IF(H22="","",I22-K22)</f>
+        <v/>
+      </c>
+      <c r="N22" s="201">
+        <f>N(B22)+N(H22)</f>
+        <v>1126410532.38</v>
+      </c>
+      <c r="O22" s="109">
+        <f>IF(N22="","",N22/N$4)</f>
+        <v>0.952008993567722</v>
+      </c>
+      <c r="P22" s="201">
+        <f>D22+IF(H22="",0,J22)</f>
+        <v>620504646.64</v>
+      </c>
+      <c r="Q22" s="109">
+        <f>P22/P$4</f>
+        <v>0.550971741082465</v>
+      </c>
+      <c r="R22" s="202">
+        <f>IF(N22="","",N22-P22)</f>
+        <v>505905885.74</v>
+      </c>
+      <c r="S22" s="203">
+        <f>IF(N22="","",O22-Q22)</f>
+        <v>0.401037252485257</v>
+      </c>
       <c r="T22" s="181" t="n"/>
       <c r="U22" s="181" t="n"/>
       <c r="V22" s="181" t="n"/>
@@ -9408,6 +9466,25 @@
       <c r="AQ26" s="181" t="n"/>
     </row>
     <row r="27">
+      <c r="A27" s="181" t="n"/>
+      <c r="B27" s="181" t="n"/>
+      <c r="C27" s="181" t="n"/>
+      <c r="D27" s="181" t="n"/>
+      <c r="E27" s="181" t="n"/>
+      <c r="F27" s="181" t="n"/>
+      <c r="G27" s="181" t="n"/>
+      <c r="H27" s="181" t="n"/>
+      <c r="I27" s="181" t="n"/>
+      <c r="J27" s="181" t="n"/>
+      <c r="K27" s="181" t="n"/>
+      <c r="L27" s="181" t="n"/>
+      <c r="M27" s="181" t="n"/>
+      <c r="N27" s="181" t="n"/>
+      <c r="O27" s="181" t="n"/>
+      <c r="P27" s="181" t="n"/>
+      <c r="Q27" s="181" t="n"/>
+      <c r="R27" s="181" t="n"/>
+      <c r="S27" s="181" t="n"/>
       <c r="T27" s="181" t="n"/>
       <c r="U27" s="181" t="n"/>
       <c r="V27" s="181" t="n"/>
@@ -9436,7 +9513,7 @@
     <row r="28">
       <c r="A28" s="204" t="n"/>
       <c r="B28" s="204">
-        <f>D21</f>
+        <f>D22</f>
         <v>620504646.64</v>
       </c>
       <c r="C28" s="204" t="n"/>
@@ -9445,8 +9522,8 @@
       <c r="F28" s="204" t="n"/>
       <c r="G28" s="204" t="n"/>
       <c r="H28" s="204">
-        <f>J21</f>
-        <v>729474678.65</v>
+        <f>J22</f>
+        <v>1007390351.99</v>
       </c>
       <c r="I28" s="204" t="n"/>
       <c r="J28" s="204" t="n"/>
@@ -9487,8 +9564,8 @@
     <row r="29">
       <c r="A29" s="204" t="n"/>
       <c r="B29" s="204">
-        <f>IF(B4="","",F4*E21)</f>
-        <v>31401350.4866053</v>
+        <f>IF(B4="","",F4*E22)</f>
+        <v>31401350.4590566</v>
       </c>
       <c r="C29" s="204" t="n"/>
       <c r="D29" s="204" t="n"/>
@@ -9496,7 +9573,7 @@
       <c r="F29" s="204" t="n"/>
       <c r="G29" s="204" t="n"/>
       <c r="H29" s="204" t="str">
-        <f>IF(H4="","",L4*K21)</f>
+        <f>IF(H4="","",L4*K22)</f>
         <v/>
       </c>
       <c r="I29" s="204" t="n"/>
@@ -9539,7 +9616,7 @@
       <c r="A30" s="204" t="n"/>
       <c r="B30" s="204">
         <f>IF(B4="","",G5*B$4)</f>
-        <v>-346066842.78151</v>
+        <v>-336531175.007532</v>
       </c>
       <c r="C30" s="204" t="n"/>
       <c r="D30" s="204" t="n"/>
@@ -9590,7 +9667,7 @@
       <c r="A31" s="204" t="n"/>
       <c r="B31" s="204">
         <f>IF(B4="","",G6*B$4)</f>
-        <v>-884263.046907184</v>
+        <v>-884263.046869816</v>
       </c>
       <c r="C31" s="204" t="n"/>
       <c r="D31" s="204" t="n"/>
@@ -9641,7 +9718,7 @@
       <c r="A32" s="204" t="n"/>
       <c r="B32" s="204">
         <f>IF(B4="","",G7*B$4)</f>
-        <v>-486861.605542351</v>
+        <v>-486861.605521777</v>
       </c>
       <c r="C32" s="204" t="n"/>
       <c r="D32" s="204" t="n"/>
@@ -9692,7 +9769,7 @@
       <c r="A33" s="204" t="n"/>
       <c r="B33" s="204">
         <f>IF(B4="","",G8*B$4)</f>
-        <v>-2675498.89610764</v>
+        <v>-2675498.89589178</v>
       </c>
       <c r="C33" s="204" t="n"/>
       <c r="D33" s="204" t="n"/>
@@ -9743,7 +9820,7 @@
       <c r="A34" s="204" t="n"/>
       <c r="B34" s="204">
         <f>IF(B4="","",G9*B$4)</f>
-        <v>128674023.794296</v>
+        <v>128674023.79738</v>
       </c>
       <c r="C34" s="204" t="n"/>
       <c r="D34" s="204" t="n"/>
@@ -9794,7 +9871,7 @@
       <c r="A35" s="204" t="n"/>
       <c r="B35" s="204">
         <f>IF(B4="","",G10*B$4)</f>
-        <v>252261678.766486</v>
+        <v>243926011.04365</v>
       </c>
       <c r="C35" s="204" t="n"/>
       <c r="D35" s="204" t="n"/>
@@ -9845,7 +9922,7 @@
       <c r="A36" s="204" t="n"/>
       <c r="B36" s="204">
         <f>IF(B4="","",G11*B$4)</f>
-        <v>-127472358.300118</v>
+        <v>-127472358.294732</v>
       </c>
       <c r="C36" s="204" t="n"/>
       <c r="D36" s="204" t="n"/>
@@ -9896,7 +9973,7 @@
       <c r="A37" s="204" t="n"/>
       <c r="B37" s="204">
         <f>IF(B4="","",G12*B$4)</f>
-        <v>-2189044.63059597</v>
+        <v>-2189044.63048418</v>
       </c>
       <c r="C37" s="204" t="n"/>
       <c r="D37" s="204" t="n"/>
@@ -9998,7 +10075,7 @@
       <c r="A39" s="204" t="n"/>
       <c r="B39" s="204">
         <f>IF(B4="","",G14*B$4)</f>
-        <v>4027369.15</v>
+        <v>2827369.14</v>
       </c>
       <c r="C39" s="204" t="n"/>
       <c r="D39" s="204" t="n"/>
@@ -10049,7 +10126,7 @@
       <c r="A40" s="204" t="n"/>
       <c r="B40" s="204">
         <f>IF(B4="","",G15*B$4)</f>
-        <v>35597311.6502615</v>
+        <v>0</v>
       </c>
       <c r="C40" s="204" t="n"/>
       <c r="D40" s="204" t="n"/>
@@ -10100,7 +10177,7 @@
       <c r="A41" s="204" t="n"/>
       <c r="B41" s="204">
         <f>IF(B4="","",G16*B$4)</f>
-        <v>179609794.412951</v>
+        <v>35597311.648718</v>
       </c>
       <c r="C41" s="204" t="n"/>
       <c r="D41" s="204" t="n"/>
@@ -10151,7 +10228,7 @@
       <c r="A42" s="204" t="n"/>
       <c r="B42" s="204">
         <f>IF(B4="","",G17*B$4)</f>
-        <v>4346889.30329168</v>
+        <v>179609794.408001</v>
       </c>
       <c r="C42" s="204" t="n"/>
       <c r="D42" s="204" t="n"/>
@@ -10202,7 +10279,7 @@
       <c r="A43" s="204" t="n"/>
       <c r="B43" s="204">
         <f>IF(B4="","",G18*B$4)</f>
-        <v>261310061.650263</v>
+        <v>4346889.30309905</v>
       </c>
       <c r="C43" s="204" t="n"/>
       <c r="D43" s="204" t="n"/>
@@ -10253,7 +10330,7 @@
       <c r="A44" s="204" t="n"/>
       <c r="B44" s="204">
         <f>IF(B4="","",G19*B$4)</f>
-        <v>-2539054.10161086</v>
+        <v>261310061.634779</v>
       </c>
       <c r="C44" s="204" t="n"/>
       <c r="D44" s="204" t="n"/>
@@ -10304,7 +10381,7 @@
       <c r="A45" s="204" t="n"/>
       <c r="B45" s="204">
         <f>IF(B4="","",G20*B$4)</f>
-        <v>-3820467.61176155</v>
+        <v>-2539054.10166784</v>
       </c>
       <c r="C45" s="204" t="n"/>
       <c r="D45" s="204" t="n"/>
@@ -10352,25 +10429,31 @@
       <c r="AQ45" s="181" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="181" t="n"/>
-      <c r="B46" s="181" t="n"/>
-      <c r="C46" s="181" t="n"/>
-      <c r="D46" s="181" t="n"/>
-      <c r="E46" s="181" t="n"/>
-      <c r="F46" s="181" t="n"/>
-      <c r="G46" s="181" t="n"/>
-      <c r="H46" s="181" t="n"/>
-      <c r="I46" s="181" t="n"/>
-      <c r="J46" s="181" t="n"/>
-      <c r="K46" s="181" t="n"/>
-      <c r="L46" s="181" t="n"/>
-      <c r="M46" s="181" t="n"/>
-      <c r="N46" s="181" t="n"/>
-      <c r="O46" s="181" t="n"/>
-      <c r="P46" s="181" t="n"/>
-      <c r="Q46" s="181" t="n"/>
-      <c r="R46" s="181" t="n"/>
-      <c r="S46" s="181" t="n"/>
+      <c r="A46" s="204" t="n"/>
+      <c r="B46" s="204">
+        <f>IF(B4="","",G21*B$4)</f>
+        <v>-3820467.61198563</v>
+      </c>
+      <c r="C46" s="204" t="n"/>
+      <c r="D46" s="204" t="n"/>
+      <c r="E46" s="204" t="n"/>
+      <c r="F46" s="204" t="n"/>
+      <c r="G46" s="204" t="n"/>
+      <c r="H46" s="204" t="str">
+        <f>IF(H4="","",M21*H$4)</f>
+        <v/>
+      </c>
+      <c r="I46" s="204" t="n"/>
+      <c r="J46" s="204" t="n"/>
+      <c r="K46" s="204" t="n"/>
+      <c r="L46" s="204" t="n"/>
+      <c r="M46" s="204" t="n"/>
+      <c r="N46" s="204" t="n"/>
+      <c r="O46" s="204" t="n"/>
+      <c r="P46" s="204" t="n"/>
+      <c r="Q46" s="204" t="n"/>
+      <c r="R46" s="204" t="n"/>
+      <c r="S46" s="204" t="n"/>
       <c r="T46" s="181" t="n"/>
       <c r="U46" s="181" t="n"/>
       <c r="V46" s="181" t="n"/>
@@ -10638,7 +10721,7 @@
         <v/>
       </c>
       <c r="E5" s="205" t="n">
-        <v>971690946.05</v>
+        <v>1250103996.52</v>
       </c>
       <c r="F5" s="136">
         <f>E5/E$5</f>
@@ -10667,11 +10750,11 @@
         <v/>
       </c>
       <c r="E6" s="209" t="n">
-        <v>560927053.33</v>
+        <v>561821896.05</v>
       </c>
       <c r="F6" s="210">
         <f>E6/E$5</f>
-        <v>0.577268992378917</v>
+        <v>0.449420126336674</v>
       </c>
       <c r="G6" s="211" t="str">
         <f>IF(C6="","",C6-E6)</f>
@@ -10699,7 +10782,7 @@
       </c>
       <c r="F7" s="210">
         <f>E7/E$5</f>
-        <v>0.000839942240192493</v>
+        <v>0.000652877098443019</v>
       </c>
       <c r="G7" s="211" t="str">
         <f>IF(C7="","",C7-E7)</f>
@@ -10727,7 +10810,7 @@
       </c>
       <c r="F8" s="210">
         <f>E8/E$5</f>
-        <v>0.000462459253970323</v>
+        <v>0.000359464069590158</v>
       </c>
       <c r="G8" s="211" t="str">
         <f>IF(C8="","",C8-E8)</f>
@@ -10755,7 +10838,7 @@
       </c>
       <c r="F9" s="210">
         <f>E9/E$5</f>
-        <v>0.0051554321673614</v>
+        <v>0.00400725601545572</v>
       </c>
       <c r="G9" s="211" t="str">
         <f>IF(C9="","",C9-E9)</f>
@@ -10783,7 +10866,7 @@
       </c>
       <c r="F10" s="210">
         <f>E10/E$5</f>
-        <v>0.0944939887247599</v>
+        <v>0.0734490518833655</v>
       </c>
       <c r="G10" s="211" t="str">
         <f>IF(C10="","",C10-E10)</f>
@@ -10811,7 +10894,7 @@
       </c>
       <c r="F11" s="210">
         <f>E11/E$5</f>
-        <v>0.27056728833251</v>
+        <v>0.210308730395131</v>
       </c>
       <c r="G11" s="211" t="str">
         <f>IF(C11="","",C11-E11)</f>
@@ -10839,7 +10922,7 @@
       </c>
       <c r="F12" s="210">
         <f>E12/E$5</f>
-        <v>0.048464191028468</v>
+        <v>0.0376706384117592</v>
       </c>
       <c r="G12" s="211" t="str">
         <f>IF(C12="","",C12-E12)</f>
@@ -10867,7 +10950,7 @@
       </c>
       <c r="F13" s="210">
         <f>E13/E$5</f>
-        <v>0.00274770587382072</v>
+        <v>0.00213575904679326</v>
       </c>
       <c r="G13" s="211" t="str">
         <f>IF(C13="","",C13-E13)</f>
@@ -10938,7 +11021,7 @@
     <row r="16" outlineLevel="1" s="12">
       <c r="B16" s="100" t="inlineStr">
         <is>
-          <t>Direct cost</t>
+          <t>М+ и сверка со сплитом</t>
         </is>
       </c>
       <c r="C16" s="209" t="n"/>
@@ -10947,11 +11030,11 @@
         <v/>
       </c>
       <c r="E16" s="209" t="n">
-        <v>-37708031.15</v>
+        <v>277518207.76</v>
       </c>
       <c r="F16" s="210">
         <f>E16/E$5</f>
-        <v>-0.0388066095534657</v>
+        <v>0.221996096750787</v>
       </c>
       <c r="G16" s="211" t="str">
         <f>IF(C16="","",C16-E16)</f>
@@ -10966,7 +11049,7 @@
     <row r="17" outlineLevel="1" s="12">
       <c r="B17" s="100" t="inlineStr">
         <is>
-          <t>PEX</t>
+          <t>Direct cost</t>
         </is>
       </c>
       <c r="C17" s="209" t="n"/>
@@ -10975,11 +11058,11 @@
         <v/>
       </c>
       <c r="E17" s="209" t="n">
-        <v>-89694325.25</v>
+        <v>-37791001.81</v>
       </c>
       <c r="F17" s="210">
         <f>E17/E$5</f>
-        <v>-0.0923074621767492</v>
+        <v>-0.0302302863723349</v>
       </c>
       <c r="G17" s="211" t="str">
         <f>IF(C17="","",C17-E17)</f>
@@ -10994,7 +11077,7 @@
     <row r="18" outlineLevel="1" s="12">
       <c r="B18" s="100" t="inlineStr">
         <is>
-          <t>Other PEX</t>
+          <t>PEX</t>
         </is>
       </c>
       <c r="C18" s="209" t="n"/>
@@ -11003,11 +11086,11 @@
         <v/>
       </c>
       <c r="E18" s="209" t="n">
-        <v>-5807323.07</v>
+        <v>-89694325.25</v>
       </c>
       <c r="F18" s="210">
         <f>E18/E$5</f>
-        <v>-0.00597651248435238</v>
+        <v>-0.0717494908421125</v>
       </c>
       <c r="G18" s="211" t="str">
         <f>IF(C18="","",C18-E18)</f>
@@ -11022,7 +11105,7 @@
     <row r="19">
       <c r="B19" s="100" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Other PEX</t>
         </is>
       </c>
       <c r="C19" s="209" t="n"/>
@@ -11031,11 +11114,11 @@
         <v/>
       </c>
       <c r="E19" s="209" t="n">
-        <v>-101498947.99</v>
+        <v>-5807323.07</v>
       </c>
       <c r="F19" s="210">
         <f>E19/E$5</f>
-        <v>-0.104455998486557</v>
+        <v>-0.00464547196566545</v>
       </c>
       <c r="G19" s="211" t="str">
         <f>IF(C19="","",C19-E19)</f>
@@ -11050,7 +11133,7 @@
     <row r="20" s="12">
       <c r="B20" s="100" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="C20" s="209" t="n"/>
@@ -11059,11 +11142,11 @@
         <v/>
       </c>
       <c r="E20" s="209" t="n">
-        <v>-1857987.23</v>
+        <v>-101647328.58</v>
       </c>
       <c r="F20" s="210">
         <f>E20/E$5</f>
-        <v>-0.00191211746651841</v>
+        <v>-0.0813110980070159</v>
       </c>
       <c r="G20" s="211" t="str">
         <f>IF(C20="","",C20-E20)</f>
@@ -11078,7 +11161,7 @@
     <row r="21">
       <c r="B21" s="100" t="inlineStr">
         <is>
-          <t>Other OPEX</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="C21" s="209" t="n"/>
@@ -11087,11 +11170,11 @@
         <v/>
       </c>
       <c r="E21" s="209" t="n">
-        <v>-5649652.71</v>
+        <v>-1857987.23</v>
       </c>
       <c r="F21" s="210">
         <f>E21/E$5</f>
-        <v>-0.005814248586926</v>
+        <v>-0.00148626613079568</v>
       </c>
       <c r="G21" s="211" t="str">
         <f>IF(C21="","",C21-E21)</f>
@@ -11104,38 +11187,65 @@
       <c r="I21" s="105" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="146" t="inlineStr">
+      <c r="B22" s="100" t="inlineStr">
+        <is>
+          <t>Other OPEX</t>
+        </is>
+      </c>
+      <c r="C22" s="209" t="n"/>
+      <c r="D22" s="210" t="str">
+        <f>IF(C22="","",C22/C$5)</f>
+        <v/>
+      </c>
+      <c r="E22" s="209" t="n">
+        <v>-5915678.59</v>
+      </c>
+      <c r="F22" s="210">
+        <f>E22/E$5</f>
+        <v>-0.00473214917036333</v>
+      </c>
+      <c r="G22" s="211" t="str">
+        <f>IF(C22="","",C22-E22)</f>
+        <v/>
+      </c>
+      <c r="H22" s="212" t="str">
+        <f>IF(C22="","",D22-F22)</f>
+        <v/>
+      </c>
+      <c r="I22" s="105" t="n"/>
+    </row>
+    <row r="23" s="12">
+      <c r="B23" s="146" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="C22" s="213" t="str">
-        <f>IF(C5="","",C5+SUM(C16:C21))</f>
-        <v/>
-      </c>
-      <c r="D22" s="214" t="str">
-        <f>IF(C22="","",C22/C$5)</f>
-        <v/>
-      </c>
-      <c r="E22" s="213">
-        <f>IF(E5="","",E5+SUM(E16:E21))</f>
-        <v>729474678.65</v>
-      </c>
-      <c r="F22" s="214">
-        <f>E22/E$5</f>
-        <v>0.750727051245431</v>
-      </c>
-      <c r="G22" s="215" t="str">
-        <f>IF(C22="","",C22-E22)</f>
-        <v/>
-      </c>
-      <c r="H22" s="216" t="str">
-        <f>IF(C22="","",D22-F22)</f>
-        <v/>
-      </c>
-      <c r="I22" s="105" t="n"/>
-    </row>
-    <row r="23"/>
+      <c r="C23" s="213" t="str">
+        <f>IF(C5="","",C5+SUM(C17:C22))</f>
+        <v/>
+      </c>
+      <c r="D23" s="214" t="str">
+        <f>IF(C23="","",C23/C$5)</f>
+        <v/>
+      </c>
+      <c r="E23" s="213">
+        <f>IF(E5="","",E5+SUM(E17:E22))</f>
+        <v>1007390351.99</v>
+      </c>
+      <c r="F23" s="214">
+        <f>E23/E$5</f>
+        <v>0.805845237511712</v>
+      </c>
+      <c r="G23" s="215" t="str">
+        <f>IF(C23="","",C23-E23)</f>
+        <v/>
+      </c>
+      <c r="H23" s="216" t="str">
+        <f>IF(C23="","",D23-F23)</f>
+        <v/>
+      </c>
+      <c r="I23" s="105" t="n"/>
+    </row>
     <row r="24" outlineLevel="1" s="12">
       <c r="B24" s="181" t="n"/>
       <c r="C24" s="181" t="n"/>
@@ -11166,7 +11276,16 @@
       <c r="H26" s="181" t="n"/>
       <c r="I26" s="181" t="n"/>
     </row>
-    <row r="27"/>
+    <row r="27">
+      <c r="B27" s="181" t="n"/>
+      <c r="C27" s="181" t="n"/>
+      <c r="D27" s="181" t="n"/>
+      <c r="E27" s="181" t="n"/>
+      <c r="F27" s="181" t="n"/>
+      <c r="G27" s="181" t="n"/>
+      <c r="H27" s="181" t="n"/>
+      <c r="I27" s="181" t="n"/>
+    </row>
     <row r="28"/>
     <row r="29"/>
     <row r="30"/>
@@ -11274,7 +11393,7 @@
         </is>
       </c>
       <c r="C5" s="205" t="n">
-        <v>1183193163.13</v>
+        <v>1183193163.08</v>
       </c>
       <c r="D5" s="136">
         <f>IF(C5="","",C5/C$5)</f>
@@ -11289,7 +11408,7 @@
       </c>
       <c r="G5" s="206">
         <f>IF(C5="","",C5-E5)</f>
-        <v>56992669.7600002</v>
+        <v>56992669.71</v>
       </c>
       <c r="H5" s="207">
         <f>IF(C5="","",D5-F5)</f>
@@ -11305,11 +11424,11 @@
         </is>
       </c>
       <c r="C6" s="209" t="n">
-        <v>457989994.88</v>
+        <v>467525662.62</v>
       </c>
       <c r="D6" s="210">
         <f>IF(C6="","",C6/C$5)</f>
-        <v>0.387079649504093</v>
+        <v>0.39513891493674</v>
       </c>
       <c r="E6" s="209" t="n">
         <v>765326605.5700001</v>
@@ -11320,11 +11439,11 @@
       </c>
       <c r="G6" s="211">
         <f>IF(C6="","",C6-E6)</f>
-        <v>-307336610.69</v>
+        <v>-297800942.95</v>
       </c>
       <c r="H6" s="212">
         <f>IF(C6="","",D6-F6)</f>
-        <v>-0.292485499042295</v>
+        <v>-0.284426233609649</v>
       </c>
       <c r="I6" s="94" t="n"/>
     </row>
@@ -11399,7 +11518,7 @@
       </c>
       <c r="D9" s="210">
         <f>IF(C9="","",C9/C$5)</f>
-        <v>0.00205589035315676</v>
+        <v>0.00205589035324364</v>
       </c>
       <c r="E9" s="209" t="n">
         <v>4861968.79</v>
@@ -11414,7 +11533,7 @@
       </c>
       <c r="H9" s="212">
         <f>IF(C9="","",D9-F9)</f>
-        <v>-0.00226125283637535</v>
+        <v>-0.00226125283628847</v>
       </c>
       <c r="I9" s="105" t="n"/>
     </row>
@@ -11429,7 +11548,7 @@
       </c>
       <c r="D10" s="210">
         <f>IF(C10="","",C10/C$5)</f>
-        <v>0.170445289217617</v>
+        <v>0.17044528922482</v>
       </c>
       <c r="E10" s="209" t="n">
         <v>69479582.98</v>
@@ -11444,7 +11563,7 @@
       </c>
       <c r="H10" s="212">
         <f>IF(C10="","",D10-F10)</f>
-        <v>0.108751493673191</v>
+        <v>0.108751493680394</v>
       </c>
       <c r="I10" s="105" t="n"/>
     </row>
@@ -11455,11 +11574,11 @@
         </is>
       </c>
       <c r="C11" s="209" t="n">
-        <v>421805564.12</v>
+        <v>413469896.39</v>
       </c>
       <c r="D11" s="210">
         <f>IF(C11="","",C11/C$5)</f>
-        <v>0.35649763475996</v>
+        <v>0.349452574010558</v>
       </c>
       <c r="E11" s="209" t="n">
         <v>161377206.43</v>
@@ -11470,11 +11589,11 @@
       </c>
       <c r="G11" s="211">
         <f>IF(C11="","",C11-E11)</f>
-        <v>260428357.69</v>
+        <v>252092689.96</v>
       </c>
       <c r="H11" s="212">
         <f>IF(C11="","",D11-F11)</f>
-        <v>0.213204138282169</v>
+        <v>0.206159077532768</v>
       </c>
       <c r="I11" s="105" t="n"/>
     </row>
@@ -11519,7 +11638,7 @@
       </c>
       <c r="D13" s="210">
         <f>IF(C13="","",C13/C$5)</f>
-        <v>0.000385584657025164</v>
+        <v>0.000385584657041458</v>
       </c>
       <c r="E13" s="209" t="n">
         <v>2517847.21</v>
@@ -11534,7 +11653,7 @@
       </c>
       <c r="H13" s="212">
         <f>IF(C13="","",D13-F13)</f>
-        <v>-0.00185011602400161</v>
+        <v>-0.00185011602398532</v>
       </c>
       <c r="I13" s="105" t="n"/>
     </row>
@@ -11549,7 +11668,7 @@
       </c>
       <c r="D14" s="210">
         <f>IF(C14="","",C14/C$5)</f>
-        <v>0.0801321377222857</v>
+        <v>0.080132137725672</v>
       </c>
       <c r="E14" s="209" t="n">
         <v>0</v>
@@ -11564,7 +11683,7 @@
       </c>
       <c r="H14" s="212">
         <f>IF(C14="","",D14-F14)</f>
-        <v>0.0801321377222857</v>
+        <v>0.080132137725672</v>
       </c>
       <c r="I14" s="105" t="n"/>
     </row>
@@ -11575,11 +11694,11 @@
         </is>
       </c>
       <c r="C15" s="209" t="n">
-        <v>4027369.15</v>
+        <v>2827369.14</v>
       </c>
       <c r="D15" s="210">
         <f>IF(C15="","",C15/C$5)</f>
-        <v>0.00340381374360384</v>
+        <v>0.00238960909192545</v>
       </c>
       <c r="E15" s="209" t="n">
         <v>0</v>
@@ -11590,227 +11709,256 @@
       </c>
       <c r="G15" s="211">
         <f>IF(C15="","",C15-E15)</f>
-        <v>4027369.15</v>
+        <v>2827369.14</v>
       </c>
       <c r="H15" s="212">
         <f>IF(C15="","",D15-F15)</f>
-        <v>0.00340381374360384</v>
+        <v>0.00238960909192545</v>
       </c>
       <c r="I15" s="105" t="n"/>
     </row>
     <row r="16" outlineLevel="1" s="12">
       <c r="B16" s="100" t="inlineStr">
         <is>
-          <t>Direct cost</t>
+          <t>М+ и сверка со сплитом</t>
         </is>
       </c>
       <c r="C16" s="209" t="n">
-        <v>-927852.26</v>
+        <v>0</v>
       </c>
       <c r="D16" s="210">
         <f>IF(C16="","",C16/C$5)</f>
-        <v>-0.000784193392011728</v>
+        <v>0</v>
       </c>
       <c r="E16" s="209" t="n">
-        <v>-34765800.63</v>
+        <v>0</v>
       </c>
       <c r="F16" s="210">
         <f>E16/E$5</f>
-        <v>-0.0308699923634096</v>
+        <v>0</v>
       </c>
       <c r="G16" s="211">
         <f>IF(C16="","",C16-E16)</f>
-        <v>33837948.37</v>
+        <v>0</v>
       </c>
       <c r="H16" s="212">
         <f>IF(C16="","",D16-F16)</f>
-        <v>0.0300857989713979</v>
+        <v>0</v>
       </c>
       <c r="I16" s="105" t="n"/>
     </row>
     <row r="17" outlineLevel="1" s="12">
       <c r="B17" s="100" t="inlineStr">
         <is>
-          <t>PEX</t>
+          <t>Direct cost</t>
         </is>
       </c>
       <c r="C17" s="209" t="n">
-        <v>62456405.7</v>
+        <v>-927852.26</v>
       </c>
       <c r="D17" s="210">
         <f>IF(C17="","",C17/C$5)</f>
-        <v>0.0527863138887473</v>
+        <v>-0.000784193392044867</v>
       </c>
       <c r="E17" s="209" t="n">
-        <v>-111510282.75</v>
+        <v>-34765800.63</v>
       </c>
       <c r="F17" s="210">
         <f>E17/E$5</f>
-        <v>-0.0990145923452056</v>
+        <v>-0.0308699923634096</v>
       </c>
       <c r="G17" s="211">
         <f>IF(C17="","",C17-E17)</f>
-        <v>173966688.45</v>
+        <v>33837948.37</v>
       </c>
       <c r="H17" s="212">
         <f>IF(C17="","",D17-F17)</f>
-        <v>0.151800906233953</v>
+        <v>0.0300857989713647</v>
       </c>
       <c r="I17" s="105" t="n"/>
     </row>
     <row r="18" outlineLevel="1" s="12">
       <c r="B18" s="100" t="inlineStr">
         <is>
-          <t>Other PEX</t>
+          <t>PEX</t>
         </is>
       </c>
       <c r="C18" s="209" t="n">
-        <v>-211306.16</v>
+        <v>62456405.7</v>
       </c>
       <c r="D18" s="210">
         <f>IF(C18="","",C18/C$5)</f>
-        <v>-0.000178589740529783</v>
+        <v>0.052786313890978</v>
       </c>
       <c r="E18" s="209" t="n">
-        <v>-4338633.91</v>
+        <v>-111510282.75</v>
       </c>
       <c r="F18" s="210">
         <f>E18/E$5</f>
-        <v>-0.00385245250338795</v>
+        <v>-0.0990145923452056</v>
       </c>
       <c r="G18" s="211">
         <f>IF(C18="","",C18-E18)</f>
-        <v>4127327.75</v>
+        <v>173966688.45</v>
       </c>
       <c r="H18" s="212">
         <f>IF(C18="","",D18-F18)</f>
-        <v>0.00367386276285817</v>
+        <v>0.151800906236184</v>
       </c>
       <c r="I18" s="105" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="100" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Other PEX</t>
         </is>
       </c>
       <c r="C19" s="209" t="n">
-        <v>-105089188</v>
+        <v>-211306.16</v>
       </c>
       <c r="D19" s="210">
         <f>IF(C19="","",C19/C$5)</f>
-        <v>-0.0888182853609454</v>
+        <v>-0.00017858974053733</v>
       </c>
       <c r="E19" s="209" t="n">
-        <v>-348750338.14</v>
+        <v>-4338633.91</v>
       </c>
       <c r="F19" s="210">
         <f>E19/E$5</f>
-        <v>-0.309669850255892</v>
+        <v>-0.00385245250338795</v>
       </c>
       <c r="G19" s="211">
         <f>IF(C19="","",C19-E19)</f>
-        <v>243661150.14</v>
+        <v>4127327.75</v>
       </c>
       <c r="H19" s="212">
         <f>IF(C19="","",D19-F19)</f>
-        <v>0.220851564894947</v>
+        <v>0.00367386276285062</v>
       </c>
       <c r="I19" s="105" t="n"/>
     </row>
     <row r="20" s="12">
       <c r="B20" s="100" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="C20" s="209" t="n">
-        <v>-3887514.7</v>
+        <v>-105089188</v>
       </c>
       <c r="D20" s="210">
         <f>IF(C20="","",C20/C$5)</f>
-        <v>-0.00328561288312048</v>
+        <v>-0.0888182853646988</v>
       </c>
       <c r="E20" s="209" t="n">
-        <v>-1283507.24</v>
+        <v>-348750338.14</v>
       </c>
       <c r="F20" s="210">
         <f>E20/E$5</f>
-        <v>-0.0011396791668589</v>
+        <v>-0.309669850255892</v>
       </c>
       <c r="G20" s="211">
         <f>IF(C20="","",C20-E20)</f>
-        <v>-2604007.46</v>
+        <v>243661150.14</v>
       </c>
       <c r="H20" s="212">
         <f>IF(C20="","",D20-F20)</f>
-        <v>-0.00214593371626158</v>
+        <v>0.220851564891194</v>
       </c>
       <c r="I20" s="105" t="n"/>
     </row>
     <row r="21">
       <c r="B21" s="100" t="inlineStr">
         <is>
-          <t>Other OPEX</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="C21" s="209" t="n">
-        <v>-9123175.279999999</v>
+        <v>-3887514.7</v>
       </c>
       <c r="D21" s="210">
         <f>IF(C21="","",C21/C$5)</f>
-        <v>-0.00771063894239018</v>
+        <v>-0.00328561288325933</v>
       </c>
       <c r="E21" s="209" t="n">
-        <v>-5047284.06</v>
+        <v>-1283507.24</v>
       </c>
       <c r="F21" s="210">
         <f>E21/E$5</f>
-        <v>-0.00448169228278057</v>
+        <v>-0.0011396791668589</v>
       </c>
       <c r="G21" s="211">
         <f>IF(C21="","",C21-E21)</f>
-        <v>-4075891.22</v>
+        <v>-2604007.46</v>
       </c>
       <c r="H21" s="212">
         <f>IF(C21="","",D21-F21)</f>
-        <v>-0.00322894665960961</v>
+        <v>-0.00214593371640043</v>
       </c>
       <c r="I21" s="105" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="146" t="inlineStr">
+      <c r="B22" s="100" t="inlineStr">
+        <is>
+          <t>Other OPEX</t>
+        </is>
+      </c>
+      <c r="C22" s="209" t="n">
+        <v>-9123175.279999999</v>
+      </c>
+      <c r="D22" s="210">
+        <f>IF(C22="","",C22/C$5)</f>
+        <v>-0.00771063894271603</v>
+      </c>
+      <c r="E22" s="209" t="n">
+        <v>-5047284.06</v>
+      </c>
+      <c r="F22" s="210">
+        <f>E22/E$5</f>
+        <v>-0.00448169228278057</v>
+      </c>
+      <c r="G22" s="211">
+        <f>IF(C22="","",C22-E22)</f>
+        <v>-4075891.22</v>
+      </c>
+      <c r="H22" s="212">
+        <f>IF(C22="","",D22-F22)</f>
+        <v>-0.00322894665993545</v>
+      </c>
+      <c r="I22" s="105" t="n"/>
+    </row>
+    <row r="23" s="12">
+      <c r="B23" s="146" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="C22" s="213">
-        <f>IF(C5="","",C5+SUM(C16:C21))</f>
-        <v>1126410532.43</v>
-      </c>
-      <c r="D22" s="214">
-        <f>IF(C22="","",C22/C$5)</f>
-        <v>0.95200899356975</v>
-      </c>
-      <c r="E22" s="213">
-        <f>IF(E5="","",E5+SUM(E16:E21))</f>
+      <c r="C23" s="213">
+        <f>IF(C5="","",C5+SUM(C17:C22))</f>
+        <v>1126410532.38</v>
+      </c>
+      <c r="D23" s="214">
+        <f>IF(C23="","",C23/C$5)</f>
+        <v>0.952008993567722</v>
+      </c>
+      <c r="E23" s="213">
+        <f>IF(E5="","",E5+SUM(E17:E22))</f>
         <v>620504646.64</v>
       </c>
-      <c r="F22" s="214">
-        <f>E22/E$5</f>
+      <c r="F23" s="214">
+        <f>E23/E$5</f>
         <v>0.550971741082465</v>
       </c>
-      <c r="G22" s="215">
-        <f>IF(C22="","",C22-E22)</f>
-        <v>505905885.79</v>
-      </c>
-      <c r="H22" s="216">
-        <f>IF(C22="","",D22-F22)</f>
-        <v>0.401037252487285</v>
-      </c>
-      <c r="I22" s="105" t="n"/>
-    </row>
-    <row r="23"/>
+      <c r="G23" s="215">
+        <f>IF(C23="","",C23-E23)</f>
+        <v>505905885.74</v>
+      </c>
+      <c r="H23" s="216">
+        <f>IF(C23="","",D23-F23)</f>
+        <v>0.401037252485257</v>
+      </c>
+      <c r="I23" s="105" t="n"/>
+    </row>
     <row r="24" outlineLevel="1" s="12">
       <c r="B24" s="181" t="n"/>
       <c r="C24" s="181" t="n"/>
@@ -11841,7 +11989,16 @@
       <c r="H26" s="181" t="n"/>
       <c r="I26" s="181" t="n"/>
     </row>
-    <row r="27"/>
+    <row r="27">
+      <c r="B27" s="181" t="n"/>
+      <c r="C27" s="181" t="n"/>
+      <c r="D27" s="181" t="n"/>
+      <c r="E27" s="181" t="n"/>
+      <c r="F27" s="181" t="n"/>
+      <c r="G27" s="181" t="n"/>
+      <c r="H27" s="181" t="n"/>
+      <c r="I27" s="181" t="n"/>
+    </row>
     <row r="28"/>
     <row r="29"/>
     <row r="30"/>
@@ -11944,7 +12101,7 @@
       </c>
       <c r="B3" s="217" t="n"/>
       <c r="C3" s="217" t="n">
-        <v>560927053.33</v>
+        <v>561821896.05</v>
       </c>
       <c r="E3" s="218" t="str">
         <f>IF(B3="","",B3-C3)</f>
@@ -12099,95 +12256,95 @@
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Gross Revenue</t>
-        </is>
-      </c>
-      <c r="B13" s="219" t="n"/>
-      <c r="C13" s="219" t="n">
-        <v>971690946.05</v>
-      </c>
-      <c r="E13" s="220" t="str">
+          <t>М+ и сверка со сплитом</t>
+        </is>
+      </c>
+      <c r="B13" s="217" t="n"/>
+      <c r="C13" s="217" t="n">
+        <v>277518207.76</v>
+      </c>
+      <c r="E13" s="218" t="str">
         <f>IF(B13="","",B13-C13)</f>
         <v/>
       </c>
-      <c r="F13" s="166" t="n"/>
-      <c r="G13" s="166" t="n"/>
+      <c r="F13" s="116" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
         <is>
+          <t>Gross Revenue</t>
+        </is>
+      </c>
+      <c r="B14" s="219" t="n"/>
+      <c r="C14" s="219" t="n">
+        <v>1250103996.52</v>
+      </c>
+      <c r="E14" s="220" t="str">
+        <f>IF(B14="","",B14-C14)</f>
+        <v/>
+      </c>
+      <c r="F14" s="166" t="n"/>
+      <c r="G14" s="166" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
           <t>Direct cost</t>
         </is>
       </c>
-      <c r="B14" s="217" t="n"/>
-      <c r="C14" s="217" t="n">
-        <v>-37708031.15</v>
-      </c>
-      <c r="E14" s="218" t="str">
-        <f>IF(B14="","",B14-C14)</f>
-        <v/>
-      </c>
-      <c r="F14" s="116" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="B15" s="217" t="n"/>
+      <c r="C15" s="217" t="n">
+        <v>-37791001.81</v>
+      </c>
+      <c r="E15" s="218" t="str">
+        <f>IF(B15="","",B15-C15)</f>
+        <v/>
+      </c>
+      <c r="F15" s="116" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>Gross margin</t>
         </is>
       </c>
-      <c r="B15" s="221" t="n"/>
-      <c r="C15" s="221" t="n">
-        <v>933982914.9</v>
-      </c>
-      <c r="E15" s="222" t="str">
-        <f>IF(B15="","",B15-C15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="17" t="inlineStr">
+      <c r="B16" s="221" t="n"/>
+      <c r="C16" s="221" t="n">
+        <v>1212312994.71</v>
+      </c>
+      <c r="E16" s="222" t="str">
+        <f>IF(B16="","",B16-C16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Gross margin %</t>
         </is>
       </c>
-      <c r="B16" s="223" t="str">
-        <f>IF(B13="","",B15/B13)</f>
-        <v/>
-      </c>
-      <c r="C16" s="223">
-        <f>IF(C13="","",C15/C13)</f>
-        <v>0.961193390446534</v>
-      </c>
-      <c r="E16" s="224" t="str">
-        <f>IF(B16="","",B16-C16)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>PEX</t>
-        </is>
-      </c>
-      <c r="B17" s="217" t="n"/>
-      <c r="C17" s="217" t="n">
-        <v>-89694325.25</v>
-      </c>
-      <c r="E17" s="218" t="str">
+      <c r="B17" s="223" t="str">
+        <f>IF(B14="","",B16/B14)</f>
+        <v/>
+      </c>
+      <c r="C17" s="223">
+        <f>IF(C14="","",C16/C14)</f>
+        <v>0.969769713627665</v>
+      </c>
+      <c r="E17" s="224" t="str">
         <f>IF(B17="","",B17-C17)</f>
         <v/>
       </c>
-      <c r="F17" s="116" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Other PEX</t>
+          <t>PEX</t>
         </is>
       </c>
       <c r="B18" s="217" t="n"/>
       <c r="C18" s="217" t="n">
-        <v>-5807323.07</v>
+        <v>-89694325.25</v>
       </c>
       <c r="E18" s="218" t="str">
         <f>IF(B18="","",B18-C18)</f>
@@ -12198,12 +12355,12 @@
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Other PEX</t>
         </is>
       </c>
       <c r="B19" s="217" t="n"/>
       <c r="C19" s="217" t="n">
-        <v>-101498947.99</v>
+        <v>-5807323.07</v>
       </c>
       <c r="E19" s="218" t="str">
         <f>IF(B19="","",B19-C19)</f>
@@ -12214,12 +12371,12 @@
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="B20" s="217" t="n"/>
       <c r="C20" s="217" t="n">
-        <v>-1857987.23</v>
+        <v>-101647328.58</v>
       </c>
       <c r="E20" s="218" t="str">
         <f>IF(B20="","",B20-C20)</f>
@@ -12230,12 +12387,12 @@
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>Other OPEX</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="B21" s="217" t="n"/>
       <c r="C21" s="217" t="n">
-        <v>-5649652.71</v>
+        <v>-1857987.23</v>
       </c>
       <c r="E21" s="218" t="str">
         <f>IF(B21="","",B21-C21)</f>
@@ -12244,95 +12401,102 @@
       <c r="F21" s="116" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="21" t="inlineStr">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>Other OPEX</t>
+        </is>
+      </c>
+      <c r="B22" s="217" t="n"/>
+      <c r="C22" s="217" t="n">
+        <v>-5915678.59</v>
+      </c>
+      <c r="E22" s="218" t="str">
+        <f>IF(B22="","",B22-C22)</f>
+        <v/>
+      </c>
+      <c r="F22" s="116" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="21" t="inlineStr">
         <is>
           <t>Total OPEX</t>
         </is>
       </c>
-      <c r="B22" s="225" t="n"/>
-      <c r="C22" s="225" t="n">
-        <v>-204508236.25</v>
-      </c>
-      <c r="E22" s="226" t="str">
-        <f>IF(B22="","",B22-C22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="19" t="inlineStr">
+      <c r="B23" s="225" t="n"/>
+      <c r="C23" s="225" t="n">
+        <v>-204922642.72</v>
+      </c>
+      <c r="E23" s="226" t="str">
+        <f>IF(B23="","",B23-C23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">EBITDA </t>
         </is>
       </c>
-      <c r="B23" s="221" t="n"/>
-      <c r="C23" s="221" t="n">
-        <v>729474678.65</v>
-      </c>
-      <c r="E23" s="222" t="str">
-        <f>IF(B23="","",B23-C23)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="28" t="inlineStr">
+      <c r="B24" s="221" t="n"/>
+      <c r="C24" s="221" t="n">
+        <v>1007390351.99</v>
+      </c>
+      <c r="E24" s="222" t="str">
+        <f>IF(B24="","",B24-C24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="28" t="inlineStr">
         <is>
           <t>EBITDA, %</t>
         </is>
       </c>
-      <c r="B24" s="227" t="str">
-        <f>IF(B13="","",B23/B13)</f>
-        <v/>
-      </c>
-      <c r="C24" s="227">
-        <f>IF(C13="","",C23/C13)</f>
-        <v>0.750727051245431</v>
-      </c>
-      <c r="D24" s="155" t="n"/>
-      <c r="E24" s="228" t="str">
-        <f>IF(B24="","",B24-C24)</f>
-        <v/>
-      </c>
-      <c r="F24" s="155" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="15" t="inlineStr">
+      <c r="B25" s="227" t="str">
+        <f>IF(B14="","",B24/B14)</f>
+        <v/>
+      </c>
+      <c r="C25" s="227">
+        <f>IF(C14="","",C24/C14)</f>
+        <v>0.805845237511712</v>
+      </c>
+      <c r="D25" s="155" t="n"/>
+      <c r="E25" s="228" t="str">
+        <f>IF(B25="","",B25-C25)</f>
+        <v/>
+      </c>
+      <c r="F25" s="155" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t>Capex</t>
         </is>
       </c>
-      <c r="B25" s="217" t="n"/>
-      <c r="C25" s="217" t="n">
+      <c r="B26" s="217" t="n"/>
+      <c r="C26" s="217" t="n">
         <v>-31696052.06</v>
       </c>
-      <c r="E25" s="218" t="str">
-        <f>IF(B25="","",B25-C25)</f>
-        <v/>
-      </c>
-      <c r="F25" s="116" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="21" t="inlineStr">
+      <c r="E26" s="218" t="str">
+        <f>IF(B26="","",B26-C26)</f>
+        <v/>
+      </c>
+      <c r="F26" s="116" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="21" t="inlineStr">
         <is>
           <t>FCF</t>
         </is>
       </c>
-      <c r="B26" s="225" t="n"/>
-      <c r="C26" s="225" t="n">
-        <v>697778626.59</v>
-      </c>
-      <c r="E26" s="226" t="str">
-        <f>IF(B26="","",B26-C26)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="181" t="n"/>
-      <c r="B27" s="181" t="n"/>
-      <c r="C27" s="181" t="n"/>
-      <c r="D27" s="181" t="n"/>
-      <c r="E27" s="181" t="n"/>
-      <c r="F27" s="181" t="n"/>
-      <c r="G27" s="181" t="n"/>
+      <c r="B27" s="225" t="n"/>
+      <c r="C27" s="225" t="n">
+        <v>975694299.9299999</v>
+      </c>
+      <c r="E27" s="226" t="str">
+        <f>IF(B27="","",B27-C27)</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="181" t="n"/>
@@ -12780,14 +12944,14 @@
         </is>
       </c>
       <c r="B3" s="217" t="n">
-        <v>457989994.88</v>
+        <v>467525662.62</v>
       </c>
       <c r="C3" s="217" t="n">
         <v>765326605.5700001</v>
       </c>
       <c r="E3" s="218">
         <f>IF(B3="","",B3-C3)</f>
-        <v>-307336610.69</v>
+        <v>-297800942.95</v>
       </c>
       <c r="F3" s="116" t="n"/>
     </row>
@@ -12870,14 +13034,14 @@
         </is>
       </c>
       <c r="B8" s="217" t="n">
-        <v>421805564.12</v>
+        <v>413469896.39</v>
       </c>
       <c r="C8" s="217" t="n">
         <v>161377206.43</v>
       </c>
       <c r="E8" s="218">
         <f>IF(B8="","",B8-C8)</f>
-        <v>260428357.69</v>
+        <v>252092689.96</v>
       </c>
       <c r="F8" s="116" t="n"/>
     </row>
@@ -12942,278 +13106,287 @@
         </is>
       </c>
       <c r="B12" s="217" t="n">
-        <v>4027369.15</v>
+        <v>2827369.14</v>
       </c>
       <c r="C12" s="217" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="218">
         <f>IF(B12="","",B12-C12)</f>
-        <v>4027369.15</v>
+        <v>2827369.14</v>
       </c>
       <c r="F12" s="116" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Gross Revenue</t>
-        </is>
-      </c>
-      <c r="B13" s="219" t="n">
-        <v>1183193163.13</v>
-      </c>
-      <c r="C13" s="219" t="n">
-        <v>1126200493.37</v>
-      </c>
-      <c r="E13" s="220">
+          <t>М+ и сверка со сплитом</t>
+        </is>
+      </c>
+      <c r="B13" s="217" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="217" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="218">
         <f>IF(B13="","",B13-C13)</f>
-        <v>56992669.7600002</v>
-      </c>
-      <c r="F13" s="166" t="n"/>
-      <c r="G13" s="166" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="F13" s="116" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
         <is>
+          <t>Gross Revenue</t>
+        </is>
+      </c>
+      <c r="B14" s="219" t="n">
+        <v>1183193163.08</v>
+      </c>
+      <c r="C14" s="219" t="n">
+        <v>1126200493.37</v>
+      </c>
+      <c r="E14" s="220">
+        <f>IF(B14="","",B14-C14)</f>
+        <v>56992669.71</v>
+      </c>
+      <c r="F14" s="166" t="n"/>
+      <c r="G14" s="166" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
           <t>Direct cost</t>
         </is>
       </c>
-      <c r="B14" s="217" t="n">
+      <c r="B15" s="217" t="n">
         <v>-927852.26</v>
       </c>
-      <c r="C14" s="217" t="n">
+      <c r="C15" s="217" t="n">
         <v>-34765800.63</v>
       </c>
-      <c r="E14" s="218">
-        <f>IF(B14="","",B14-C14)</f>
+      <c r="E15" s="218">
+        <f>IF(B15="","",B15-C15)</f>
         <v>33837948.37</v>
       </c>
-      <c r="F14" s="116" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="F15" s="116" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>Gross margin</t>
         </is>
       </c>
-      <c r="B15" s="221" t="n">
-        <v>1182265310.87</v>
-      </c>
-      <c r="C15" s="221" t="n">
+      <c r="B16" s="221" t="n">
+        <v>1182265310.82</v>
+      </c>
+      <c r="C16" s="221" t="n">
         <v>1091434692.74</v>
       </c>
-      <c r="E15" s="222">
-        <f>IF(B15="","",B15-C15)</f>
-        <v>90830618.1299999</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="17" t="inlineStr">
+      <c r="E16" s="222">
+        <f>IF(B16="","",B16-C16)</f>
+        <v>90830618.0799999</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Gross margin %</t>
         </is>
       </c>
-      <c r="B16" s="223">
-        <f>IF(B13="","",B15/B13)</f>
-        <v>0.999215806607988</v>
-      </c>
-      <c r="C16" s="223">
-        <f>IF(C13="","",C15/C13)</f>
+      <c r="B17" s="223">
+        <f>IF(B14="","",B16/B14)</f>
+        <v>0.999215806607955</v>
+      </c>
+      <c r="C17" s="223">
+        <f>IF(C14="","",C16/C14)</f>
         <v>0.969130007636591</v>
       </c>
-      <c r="E16" s="224">
-        <f>IF(B16="","",B16-C16)</f>
-        <v>0.0300857989713975</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>PEX</t>
-        </is>
-      </c>
-      <c r="B17" s="217" t="n">
-        <v>62456405.7</v>
-      </c>
-      <c r="C17" s="217" t="n">
-        <v>-111510282.75</v>
-      </c>
-      <c r="E17" s="218">
+      <c r="E17" s="224">
         <f>IF(B17="","",B17-C17)</f>
-        <v>173966688.45</v>
-      </c>
-      <c r="F17" s="116" t="n"/>
+        <v>0.0300857989713647</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Other PEX</t>
+          <t>PEX</t>
         </is>
       </c>
       <c r="B18" s="217" t="n">
-        <v>-211306.16</v>
+        <v>62456405.7</v>
       </c>
       <c r="C18" s="217" t="n">
-        <v>-4338633.91</v>
+        <v>-111510282.75</v>
       </c>
       <c r="E18" s="218">
         <f>IF(B18="","",B18-C18)</f>
-        <v>4127327.75</v>
+        <v>173966688.45</v>
       </c>
       <c r="F18" s="116" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Other PEX</t>
         </is>
       </c>
       <c r="B19" s="217" t="n">
-        <v>-105089188</v>
+        <v>-211306.16</v>
       </c>
       <c r="C19" s="217" t="n">
-        <v>-348750338.14</v>
+        <v>-4338633.91</v>
       </c>
       <c r="E19" s="218">
         <f>IF(B19="","",B19-C19)</f>
-        <v>243661150.14</v>
+        <v>4127327.75</v>
       </c>
       <c r="F19" s="116" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="B20" s="217" t="n">
-        <v>-3887514.7</v>
+        <v>-105089188</v>
       </c>
       <c r="C20" s="217" t="n">
-        <v>-1283507.24</v>
+        <v>-348750338.14</v>
       </c>
       <c r="E20" s="218">
         <f>IF(B20="","",B20-C20)</f>
-        <v>-2604007.46</v>
+        <v>243661150.14</v>
       </c>
       <c r="F20" s="116" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>Other OPEX</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="B21" s="217" t="n">
-        <v>-9123175.279999999</v>
+        <v>-3887514.7</v>
       </c>
       <c r="C21" s="217" t="n">
-        <v>-5047284.06</v>
+        <v>-1283507.24</v>
       </c>
       <c r="E21" s="218">
         <f>IF(B21="","",B21-C21)</f>
+        <v>-2604007.46</v>
+      </c>
+      <c r="F21" s="116" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>Other OPEX</t>
+        </is>
+      </c>
+      <c r="B22" s="217" t="n">
+        <v>-9123175.279999999</v>
+      </c>
+      <c r="C22" s="217" t="n">
+        <v>-5047284.06</v>
+      </c>
+      <c r="E22" s="218">
+        <f>IF(B22="","",B22-C22)</f>
         <v>-4075891.22</v>
       </c>
-      <c r="F21" s="116" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="21" t="inlineStr">
+      <c r="F22" s="116" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="21" t="inlineStr">
         <is>
           <t>Total OPEX</t>
         </is>
       </c>
-      <c r="B22" s="225" t="n">
+      <c r="B23" s="225" t="n">
         <v>-55854778.45</v>
       </c>
-      <c r="C22" s="225" t="n">
+      <c r="C23" s="225" t="n">
         <v>-470930046.1</v>
       </c>
-      <c r="E22" s="226">
-        <f>IF(B22="","",B22-C22)</f>
+      <c r="E23" s="226">
+        <f>IF(B23="","",B23-C23)</f>
         <v>415075267.65</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="19" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">EBITDA </t>
         </is>
       </c>
-      <c r="B23" s="221" t="n">
-        <v>1126410532.42</v>
-      </c>
-      <c r="C23" s="221" t="n">
+      <c r="B24" s="221" t="n">
+        <v>1126410532.37</v>
+      </c>
+      <c r="C24" s="221" t="n">
         <v>620504646.64</v>
       </c>
-      <c r="E23" s="222">
-        <f>IF(B23="","",B23-C23)</f>
-        <v>505905885.78</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="28" t="inlineStr">
+      <c r="E24" s="222">
+        <f>IF(B24="","",B24-C24)</f>
+        <v>505905885.73</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="28" t="inlineStr">
         <is>
           <t>EBITDA, %</t>
         </is>
       </c>
-      <c r="B24" s="227">
-        <f>IF(B13="","",B23/B13)</f>
-        <v>0.952008993561298</v>
-      </c>
-      <c r="C24" s="227">
-        <f>IF(C13="","",C23/C13)</f>
+      <c r="B25" s="227">
+        <f>IF(B14="","",B24/B14)</f>
+        <v>0.95200899355927</v>
+      </c>
+      <c r="C25" s="227">
+        <f>IF(C14="","",C24/C14)</f>
         <v>0.550971741082465</v>
       </c>
-      <c r="D24" s="155" t="n"/>
-      <c r="E24" s="228">
-        <f>IF(B24="","",B24-C24)</f>
-        <v>0.401037252478833</v>
-      </c>
-      <c r="F24" s="155" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="15" t="inlineStr">
+      <c r="D25" s="155" t="n"/>
+      <c r="E25" s="228">
+        <f>IF(B25="","",B25-C25)</f>
+        <v>0.401037252476805</v>
+      </c>
+      <c r="F25" s="155" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t>Capex</t>
         </is>
       </c>
-      <c r="B25" s="217" t="n">
+      <c r="B26" s="217" t="n">
         <v>-185765416.81</v>
       </c>
-      <c r="C25" s="217" t="n">
+      <c r="C26" s="217" t="n">
         <v>-242709711.72</v>
       </c>
-      <c r="E25" s="218">
-        <f>IF(B25="","",B25-C25)</f>
+      <c r="E26" s="218">
+        <f>IF(B26="","",B26-C26)</f>
         <v>56944294.91</v>
       </c>
-      <c r="F25" s="116" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="21" t="inlineStr">
+      <c r="F26" s="116" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="21" t="inlineStr">
         <is>
           <t>FCF</t>
         </is>
       </c>
-      <c r="B26" s="225" t="n">
-        <v>940645115.61</v>
-      </c>
-      <c r="C26" s="225" t="n">
+      <c r="B27" s="225" t="n">
+        <v>940645115.5599999</v>
+      </c>
+      <c r="C27" s="225" t="n">
         <v>377794934.93</v>
       </c>
-      <c r="E26" s="226">
-        <f>IF(B26="","",B26-C26)</f>
-        <v>562850180.68</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="181" t="n"/>
-      <c r="B27" s="181" t="n"/>
-      <c r="C27" s="181" t="n"/>
-      <c r="D27" s="181" t="n"/>
-      <c r="E27" s="181" t="n"/>
-      <c r="F27" s="181" t="n"/>
-      <c r="G27" s="181" t="n"/>
+      <c r="E27" s="226">
+        <f>IF(B27="","",B27-C27)</f>
+        <v>562850180.63</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="181" t="n"/>

</xml_diff>